<commit_message>
Audit 3 page fixes: interactive donor-web counts, vendor bars, guide wording, card order
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BHR3oVojTDcQacx4y1dmUd
</commit_message>
<xml_diff>
--- a/data/whos-buying-pdx-data.xlsx
+++ b/data/whos-buying-pdx-data.xlsx
@@ -204,7 +204,7 @@
     <t xml:space="preserve">Gave to a Republican campaign in 2024–2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Gave to two or more of the six candidates</t>
+    <t xml:space="preserve">Matched for two or more of the six candidates (a Republican match on each one's list)</t>
   </si>
   <si>
     <t xml:space="preserve">Rest only on a link through other filings (no direct address or ZIP + employer match)</t>
@@ -262,7 +262,7 @@
     <t xml:space="preserve">Several Drazan gifts were filed under a nickname or another form of the donor's name.</t>
   </si>
   <si>
-    <t xml:space="preserve">Gave to two or more of the six</t>
+    <t xml:space="preserve">Matched for two or more of the six</t>
   </si>
   <si>
     <t xml:space="preserve">was 53</t>

</xml_diff>